<commit_message>
form tables of contribution of body dissatisfaction in explaining BP3 levels
</commit_message>
<xml_diff>
--- a/mapping_regression_formulas_and_equation_numbers.xlsx
+++ b/mapping_regression_formulas_and_equation_numbers.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vynguyen/Dropbox/Mac/Documents/GitHub/weight_perception_bp3/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1849EBB2-B328-DB41-AF03-CE6685B2C340}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7412A567-EDCE-9442-9A16-ACF77AFF65E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28800" yWindow="500" windowWidth="40960" windowHeight="22540" xr2:uid="{EA8BF802-6658-9144-8C73-C0DC3C33AB58}"/>
+    <workbookView xWindow="69780" yWindow="1840" windowWidth="40960" windowHeight="22540" xr2:uid="{EA8BF802-6658-9144-8C73-C0DC3C33AB58}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,35 +36,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="15">
   <si>
     <t>regression_formula</t>
   </si>
   <si>
-    <t>log10(URXBP3) ~ race + RIDAGEYR + SDDSRVYR + URXUCR + BMXBMI + INDFMPIR</t>
-  </si>
-  <si>
-    <t>log10(URXBP3) ~ race + RIDAGEYR + SDDSRVYR + URXUCR + BMXBMI + INDFMPIR + weight_perception</t>
-  </si>
-  <si>
-    <t>log10(URXBP3) ~ race + RIDAGEYR + SDDSRVYR + URXUCR + BMXBMI + INDFMPIR + sunscreen_usage_ordinal</t>
-  </si>
-  <si>
-    <t>log10(URXBP3) ~ race + RIDAGEYR + SDDSRVYR + URXUCR + BMXBMI + INDFMPIR + sunscreen_usage_ordinal + weight_perception</t>
-  </si>
-  <si>
-    <t>log10(URXBP3) ~ RIDAGEYR + SDDSRVYR + URXUCR + BMXBMI + INDFMPIR</t>
-  </si>
-  <si>
-    <t>log10(URXBP3) ~ RIDAGEYR + SDDSRVYR + URXUCR + BMXBMI + INDFMPIR + race_weight_perception</t>
-  </si>
-  <si>
-    <t>log10(URXBP3) ~ RIDAGEYR + SDDSRVYR + URXUCR + BMXBMI + INDFMPIR + sunscreen_usage_ordinal</t>
-  </si>
-  <si>
-    <t>log10(URXBP3) ~ RIDAGEYR + SDDSRVYR + URXUCR + BMXBMI + INDFMPIR + sunscreen_usage_ordinal + race_weight_perception</t>
-  </si>
-  <si>
     <t>equation_number</t>
   </si>
   <si>
@@ -87,6 +63,24 @@
   </si>
   <si>
     <t>Race/ethnicity</t>
+  </si>
+  <si>
+    <t>log10(URXBP3) ~ race + RIDAGEYR + SDDSRVYR + URXUCR + BMXBMI + INDFMPIR</t>
+  </si>
+  <si>
+    <t>log10(URXBP3) ~ race + RIDAGEYR + SDDSRVYR + URXUCR + BMXBMI + INDFMPIR + weight_perception</t>
+  </si>
+  <si>
+    <t>log10(URXBP3) ~ race + RIDAGEYR + SDDSRVYR + URXUCR + BMXBMI + INDFMPIR + sunscreen_usage_ordinal</t>
+  </si>
+  <si>
+    <t>log10(URXBP3) ~ race + RIDAGEYR + SDDSRVYR + URXUCR + BMXBMI + INDFMPIR + sunscreen_usage_ordinal + weight_perception</t>
+  </si>
+  <si>
+    <t>log10(URXBP3) ~ RIDAGEYR + SDDSRVYR + URXUCR + BMXBMI + INDFMPIR + race_weight_perception</t>
+  </si>
+  <si>
+    <t>log10(URXBP3) ~ RIDAGEYR + SDDSRVYR + URXUCR + BMXBMI + INDFMPIR + sunscreen_usage_ordinal + race_weight_perception</t>
   </si>
 </sst>
 </file>
@@ -471,7 +465,7 @@
   <cols>
     <col min="1" max="1" width="121.83203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="15.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="33.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:19" s="4" customFormat="1" x14ac:dyDescent="0.2">
@@ -479,21 +473,21 @@
         <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
     </row>
     <row r="2" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="B2" s="5">
         <v>1</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
@@ -513,13 +507,13 @@
     </row>
     <row r="3" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="B3" s="5">
         <v>1</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="D3" s="3"/>
       <c r="E3" s="3"/>
@@ -539,13 +533,13 @@
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="B4" s="5">
         <v>4</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
@@ -565,13 +559,13 @@
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="B5" s="5">
         <v>4</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="D5" s="3"/>
       <c r="E5" s="3"/>
@@ -591,13 +585,13 @@
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="B6" s="5">
         <v>2</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="D6" s="1"/>
       <c r="E6" s="1"/>
@@ -617,13 +611,13 @@
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="B7" s="5">
         <v>2</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="D7" s="3"/>
       <c r="E7" s="3"/>
@@ -643,13 +637,13 @@
     </row>
     <row r="8" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="B8" s="5">
         <v>5</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
@@ -669,13 +663,13 @@
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="B9" s="5">
         <v>5</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="D9" s="3"/>
       <c r="E9" s="3"/>
@@ -695,13 +689,13 @@
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="B10" s="5">
         <v>7</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="D10" s="1"/>
       <c r="E10" s="1"/>
@@ -721,13 +715,13 @@
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="B11" s="5">
         <v>7</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="D11" s="3"/>
       <c r="E11" s="3"/>
@@ -747,13 +741,13 @@
     </row>
     <row r="12" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="B12" s="5">
         <v>8</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="D12" s="1"/>
       <c r="E12" s="1"/>
@@ -773,13 +767,13 @@
     </row>
     <row r="13" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="B13" s="5">
         <v>8</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="D13" s="3"/>
       <c r="E13" s="3"/>

</xml_diff>